<commit_message>
Updated till January 2026
</commit_message>
<xml_diff>
--- a/data/Crop_Anuarios_JA.xlsx
+++ b/data/Crop_Anuarios_JA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucordoba-my.sharepoint.com/personal/b42otmoj_uco_es/Documents/Trabajo/PROYECTOS ON/2013_2021 DEOLEO/MODEL/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="304" documentId="13_ncr:4000b_{6F0A6980-1E43-4129-9F59-D808CC2AE339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71154937-2EFA-4CDB-988C-3CFC03205B22}"/>
+  <xr:revisionPtr revIDLastSave="343" documentId="13_ncr:4000b_{6F0A6980-1E43-4129-9F59-D808CC2AE339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D9F6654-64B6-4098-A120-1A4B0712BE45}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="653" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="653" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Crop" sheetId="2" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>Year</t>
   </si>
@@ -203,6 +203,9 @@
   </si>
   <si>
     <t>2024_2025</t>
+  </si>
+  <si>
+    <t>2025_2026</t>
   </si>
 </sst>
 </file>
@@ -308,7 +311,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -325,7 +328,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Excel Built-in Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -773,7 +779,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="10.7109375" style="1"/>
@@ -781,14 +787,11 @@
     <col min="6" max="6" width="13" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" style="1"/>
     <col min="8" max="8" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="10.7109375" style="1"/>
-    <col min="12" max="12" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="10.7109375" style="1"/>
+    <col min="9" max="9" width="11.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -814,7 +817,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1982</v>
       </c>
@@ -828,7 +831,7 @@
         <v>504643</v>
       </c>
       <c r="E2" s="4">
-        <f t="shared" ref="E2:E44" si="0">D2*100/C2</f>
+        <f t="shared" ref="E2:E45" si="0">D2*100/C2</f>
         <v>21.153838092611206</v>
       </c>
       <c r="F2" s="3">
@@ -838,12 +841,11 @@
         <v>666134</v>
       </c>
       <c r="H2" s="4">
-        <f t="shared" ref="H2:H44" si="1">G2*100/F2</f>
+        <f t="shared" ref="H2:H45" si="1">G2*100/F2</f>
         <v>21.706660583941606</v>
       </c>
-      <c r="I2" s="8"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1983</v>
       </c>
@@ -870,9 +872,8 @@
         <f t="shared" si="1"/>
         <v>21.263867957002645</v>
       </c>
-      <c r="I3" s="8"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>1984</v>
       </c>
@@ -899,9 +900,8 @@
         <f t="shared" si="1"/>
         <v>21.711650755399017</v>
       </c>
-      <c r="I4" s="8"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>1985</v>
       </c>
@@ -928,9 +928,8 @@
         <f t="shared" si="1"/>
         <v>21.184276494746385</v>
       </c>
-      <c r="I5" s="8"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>1986</v>
       </c>
@@ -957,9 +956,8 @@
         <f t="shared" si="1"/>
         <v>21.121086675291075</v>
       </c>
-      <c r="I6" s="8"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>1987</v>
       </c>
@@ -986,9 +984,8 @@
         <f t="shared" si="1"/>
         <v>20.029920013103656</v>
       </c>
-      <c r="I7" s="8"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>1988</v>
       </c>
@@ -1015,9 +1012,8 @@
         <f t="shared" si="1"/>
         <v>19.44027453271028</v>
       </c>
-      <c r="I8" s="8"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>1989</v>
       </c>
@@ -1044,9 +1040,8 @@
         <f t="shared" si="1"/>
         <v>20.695449592304513</v>
       </c>
-      <c r="I9" s="8"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>1990</v>
       </c>
@@ -1073,9 +1068,8 @@
         <f t="shared" si="1"/>
         <v>20.277654446276799</v>
       </c>
-      <c r="I10" s="8"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>1991</v>
       </c>
@@ -1102,9 +1096,8 @@
         <f t="shared" si="1"/>
         <v>21.75724664269465</v>
       </c>
-      <c r="I11" s="8"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>1992</v>
       </c>
@@ -1131,9 +1124,8 @@
         <f t="shared" si="1"/>
         <v>21.151503835969855</v>
       </c>
-      <c r="I12" s="8"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>1993</v>
       </c>
@@ -1160,9 +1152,8 @@
         <f t="shared" si="1"/>
         <v>21.071650612119583</v>
       </c>
-      <c r="I13" s="8"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>1994</v>
       </c>
@@ -1189,9 +1180,8 @@
         <f t="shared" si="1"/>
         <v>20.202338957055215</v>
       </c>
-      <c r="I14" s="8"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>1995</v>
       </c>
@@ -1218,9 +1208,8 @@
         <f t="shared" si="1"/>
         <v>21.076594842669952</v>
       </c>
-      <c r="I15" s="8"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>1996</v>
       </c>
@@ -1247,9 +1236,8 @@
         <f t="shared" si="1"/>
         <v>22.044405424762608</v>
       </c>
-      <c r="I16" s="8"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>1997</v>
       </c>
@@ -1276,9 +1264,8 @@
         <f t="shared" si="1"/>
         <v>20.120476737507179</v>
       </c>
-      <c r="I17" s="8"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>1998</v>
       </c>
@@ -1305,9 +1292,8 @@
         <f t="shared" si="1"/>
         <v>21.345658355938841</v>
       </c>
-      <c r="I18" s="8"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>1999</v>
       </c>
@@ -1334,9 +1320,8 @@
         <f t="shared" si="1"/>
         <v>21.994596375617792</v>
       </c>
-      <c r="I19" s="8"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>2000</v>
       </c>
@@ -1363,9 +1348,8 @@
         <f t="shared" si="1"/>
         <v>20.796430610475568</v>
       </c>
-      <c r="I20" s="8"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>2001</v>
       </c>
@@ -1392,9 +1376,8 @@
         <f t="shared" si="1"/>
         <v>21.888911122741128</v>
       </c>
-      <c r="I21" s="8"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>2002</v>
       </c>
@@ -1421,9 +1404,8 @@
         <f t="shared" si="1"/>
         <v>20.628592556075919</v>
       </c>
-      <c r="I22" s="8"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>2003</v>
       </c>
@@ -1450,9 +1432,8 @@
         <f t="shared" si="1"/>
         <v>20.539340335360237</v>
       </c>
-      <c r="I23" s="8"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>2004</v>
       </c>
@@ -1479,9 +1460,8 @@
         <f t="shared" si="1"/>
         <v>21.191691607300932</v>
       </c>
-      <c r="I24" s="8"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>2005</v>
       </c>
@@ -1508,9 +1488,8 @@
         <f t="shared" si="1"/>
         <v>22.472856738925284</v>
       </c>
-      <c r="I25" s="8"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>2006</v>
       </c>
@@ -1537,9 +1516,8 @@
         <f t="shared" si="1"/>
         <v>20.680118371978359</v>
       </c>
-      <c r="I26" s="8"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>2007</v>
       </c>
@@ -1566,9 +1544,8 @@
         <f t="shared" si="1"/>
         <v>20.917768257385237</v>
       </c>
-      <c r="I27" s="8"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>2008</v>
       </c>
@@ -1595,9 +1572,8 @@
         <f t="shared" si="1"/>
         <v>20.856615224899677</v>
       </c>
-      <c r="I28" s="8"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>2009</v>
       </c>
@@ -1624,9 +1600,8 @@
         <f t="shared" si="1"/>
         <v>21.354951605235204</v>
       </c>
-      <c r="I29" s="8"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>2010</v>
       </c>
@@ -1653,9 +1628,8 @@
         <f t="shared" si="1"/>
         <v>20.880097587417197</v>
       </c>
-      <c r="I30" s="8"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>2011</v>
       </c>
@@ -1682,9 +1656,8 @@
         <f t="shared" si="1"/>
         <v>21.319020762041465</v>
       </c>
-      <c r="I31" s="8"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>2012</v>
       </c>
@@ -1711,9 +1684,8 @@
         <f t="shared" si="1"/>
         <v>18.926078085908184</v>
       </c>
-      <c r="I32" s="8"/>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>2013</v>
       </c>
@@ -1740,9 +1712,8 @@
         <f t="shared" si="1"/>
         <v>20.135368306482899</v>
       </c>
-      <c r="I33" s="8"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>2014</v>
       </c>
@@ -1769,9 +1740,8 @@
         <f t="shared" si="1"/>
         <v>20.300768964858719</v>
       </c>
-      <c r="I34" s="8"/>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>2015</v>
       </c>
@@ -1798,9 +1768,8 @@
         <f t="shared" si="1"/>
         <v>20.419031562430678</v>
       </c>
-      <c r="I35" s="8"/>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>2016</v>
       </c>
@@ -1827,9 +1796,8 @@
         <f t="shared" si="1"/>
         <v>19.504710391713946</v>
       </c>
-      <c r="I36" s="8"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>2017</v>
       </c>
@@ -1856,9 +1824,8 @@
         <f t="shared" si="1"/>
         <v>20.491994891845465</v>
       </c>
-      <c r="I37" s="8"/>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>2018</v>
       </c>
@@ -1885,9 +1852,8 @@
         <f t="shared" si="1"/>
         <v>19.324324499359708</v>
       </c>
-      <c r="I38" s="8"/>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>2019</v>
       </c>
@@ -1914,9 +1880,8 @@
         <f t="shared" si="1"/>
         <v>20.592809873747555</v>
       </c>
-      <c r="I39" s="8"/>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>2020</v>
       </c>
@@ -1943,9 +1908,8 @@
         <f t="shared" si="1"/>
         <v>18.085525252025278</v>
       </c>
-      <c r="I40" s="8"/>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>2021</v>
       </c>
@@ -1972,9 +1936,8 @@
         <f t="shared" si="1"/>
         <v>19.780843165849131</v>
       </c>
-      <c r="I41" s="8"/>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>2022</v>
       </c>
@@ -2001,9 +1964,8 @@
         <f t="shared" si="1"/>
         <v>19.026808968406748</v>
       </c>
-      <c r="I42" s="8"/>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>2023</v>
       </c>
@@ -2011,28 +1973,27 @@
         <v>55</v>
       </c>
       <c r="C43" s="3">
-        <v>3340527</v>
+        <v>3079922</v>
       </c>
       <c r="D43" s="3">
         <v>576617</v>
       </c>
       <c r="E43" s="4">
         <f t="shared" si="0"/>
-        <v>17.26125847807846</v>
+        <v>18.721805292471693</v>
       </c>
       <c r="F43" s="3">
-        <v>4749700</v>
+        <v>4627976</v>
       </c>
       <c r="G43" s="3">
-        <v>835584</v>
+        <v>843371</v>
       </c>
       <c r="H43" s="4">
         <f t="shared" si="1"/>
-        <v>17.592353201254816</v>
-      </c>
-      <c r="I43" s="8"/>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+        <v>18.223322679287879</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>2024</v>
       </c>
@@ -2059,11 +2020,38 @@
         <f t="shared" si="1"/>
         <v>18.056349410462872</v>
       </c>
-      <c r="I44" s="8"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="3">
+        <v>2025</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C45" s="8">
+        <v>5372249</v>
+      </c>
+      <c r="D45" s="8">
+        <v>878376</v>
+      </c>
+      <c r="E45" s="8">
+        <f t="shared" si="0"/>
+        <v>16.350247354506465</v>
+      </c>
+      <c r="F45" s="9">
+        <v>7027959</v>
+      </c>
+      <c r="G45" s="8">
+        <v>1184927</v>
+      </c>
+      <c r="H45" s="8">
+        <f t="shared" si="1"/>
+        <v>16.860186577639396</v>
+      </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I44">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H44">
     <sortCondition ref="A4:A44"/>
   </sortState>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>